<commit_message>
Updates on README and Deleted Old version Q input py
</commit_message>
<xml_diff>
--- a/result_sentiment_adjusted_Q/evaluation_metrics.xlsx
+++ b/result_sentiment_adjusted_Q/evaluation_metrics.xlsx
@@ -441,17 +441,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Sentiment BL (Baseline Omega)</t>
+          <t>RAW Sentiment BL (Baseline Omega)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Sentiment BL (Advanced Omega)</t>
+          <t>RAW Sentiment BL (Advanced Omega)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Sentiment Dynamic BL</t>
+          <t>RAW Sentiment Dynamic BL</t>
         </is>
       </c>
     </row>
@@ -462,19 +462,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1807271344036079</v>
+        <v>0.1807271374065327</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4331300178292418</v>
+        <v>0.4331299891482575</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2201005012310898</v>
+        <v>0.2201005070173749</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2392680792094109</v>
+        <v>0.2392681540663875</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2352873825885871</v>
+        <v>0.2352874789007391</v>
       </c>
     </row>
     <row r="3">
@@ -484,19 +484,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.076066752993368</v>
+        <v>1.076066663596196</v>
       </c>
       <c r="C3" t="n">
-        <v>1.250937387120761</v>
+        <v>1.250937268983203</v>
       </c>
       <c r="D3" t="n">
-        <v>1.154997036985717</v>
+        <v>1.154997069518551</v>
       </c>
       <c r="E3" t="n">
-        <v>1.176625388335971</v>
+        <v>1.176625662700239</v>
       </c>
       <c r="F3" t="n">
-        <v>1.044729702475751</v>
+        <v>1.044729925675667</v>
       </c>
     </row>
     <row r="4">
@@ -507,16 +507,16 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>0.9907966282521912</v>
+        <v>0.9907964388844448</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6678530320145066</v>
+        <v>0.6678531353588788</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7172828369038098</v>
+        <v>0.7172838556096787</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4845517329248966</v>
+        <v>0.4845525786168947</v>
       </c>
     </row>
     <row r="5">
@@ -526,19 +526,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.2028773863168427</v>
+        <v>-0.2028774508884138</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.452530631002677</v>
+        <v>-0.4525306064401637</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.2780680754738878</v>
+        <v>-0.2780681999688465</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.3089628860330432</v>
+        <v>-0.3089628874726069</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.3553682997090751</v>
+        <v>-0.3553683785948052</v>
       </c>
     </row>
     <row r="6">
@@ -548,19 +548,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.167951601423301</v>
+        <v>0.1679516181669876</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3462443622587396</v>
+        <v>0.3462443720301961</v>
       </c>
       <c r="D6" t="n">
-        <v>0.190563693397433</v>
+        <v>0.1905636930396036</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2033511103714947</v>
+        <v>0.2033511265743524</v>
       </c>
       <c r="F6" t="n">
-        <v>0.225213643329001</v>
+        <v>0.2252136874021003</v>
       </c>
     </row>
     <row r="7">
@@ -570,19 +570,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0737089452488867</v>
+        <v>-0.07370896689482442</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.1207384822071983</v>
+        <v>-0.1207385826560214</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.08182216831353969</v>
+        <v>-0.08182223506434683</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.08710519545995069</v>
+        <v>-0.08710519410966466</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.09738185072464102</v>
+        <v>-0.09738182847686389</v>
       </c>
     </row>
     <row r="8">
@@ -595,16 +595,16 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6380535544738818</v>
+        <v>0.6380536831046097</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06139300902410207</v>
+        <v>0.06139298543065741</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1572399172977312</v>
+        <v>0.1572397642942774</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3767784543333612</v>
+        <v>0.3767782789755982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed backtest start date error in backtest sentiment adjusted Q
</commit_message>
<xml_diff>
--- a/result_sentiment_adjusted_Q/evaluation_metrics.xlsx
+++ b/result_sentiment_adjusted_Q/evaluation_metrics.xlsx
@@ -462,19 +462,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1807271374065327</v>
+        <v>0.1710126995111861</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4331299891482575</v>
+        <v>0.4049178582871612</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2201005070173749</v>
+        <v>0.1939703894627932</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2392681540663875</v>
+        <v>0.214624140535691</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2352874789007391</v>
+        <v>0.2193739831441971</v>
       </c>
     </row>
     <row r="3">
@@ -484,19 +484,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.076066663596196</v>
+        <v>1.144890112258371</v>
       </c>
       <c r="C3" t="n">
-        <v>1.250937268983203</v>
+        <v>1.160894442697566</v>
       </c>
       <c r="D3" t="n">
-        <v>1.154997069518551</v>
+        <v>1.080989801407628</v>
       </c>
       <c r="E3" t="n">
-        <v>1.176625662700239</v>
+        <v>1.132898509608024</v>
       </c>
       <c r="F3" t="n">
-        <v>1.044729925675667</v>
+        <v>1.126472658581236</v>
       </c>
     </row>
     <row r="4">
@@ -507,16 +507,16 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>0.9907964388844448</v>
+        <v>0.8936043986040845</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6678531353588788</v>
+        <v>0.414883048441232</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7172838556096787</v>
+        <v>0.5996862667152726</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4845525786168947</v>
+        <v>0.5399633801994974</v>
       </c>
     </row>
     <row r="5">
@@ -526,19 +526,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.2028774508884138</v>
+        <v>-0.2028774012753196</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.4525306064401637</v>
+        <v>-0.4525305106667451</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.2780681999688465</v>
+        <v>-0.2715310900557988</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.3089628874726069</v>
+        <v>-0.2984331714520753</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.3553683785948052</v>
+        <v>-0.2753185598698785</v>
       </c>
     </row>
     <row r="6">
@@ -548,19 +548,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1679516181669876</v>
+        <v>0.1493704047926943</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3462443720301961</v>
+        <v>0.3487981709570898</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1905636930396036</v>
+        <v>0.1794377608467828</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2033511265743524</v>
+        <v>0.1894469263711449</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2252136874021003</v>
+        <v>0.1947441701962772</v>
       </c>
     </row>
     <row r="7">
@@ -570,19 +570,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.07370896689482442</v>
+        <v>-0.05269718626937447</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.1207385826560214</v>
+        <v>-0.1272865239573453</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.08182223506434683</v>
+        <v>-0.0628198079366271</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.08710519410966466</v>
+        <v>-0.07467974982778716</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.09738182847686389</v>
+        <v>-0.08837081905292817</v>
       </c>
     </row>
     <row r="8">
@@ -595,16 +595,16 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.6380536831046097</v>
+        <v>0.710015972005132</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06139298543065741</v>
+        <v>0.08432804632459089</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1572397642942774</v>
+        <v>0.1561427992380214</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3767782789755982</v>
+        <v>0.3434836760998189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>